<commit_message>
thuật ngữ: "Nguyên bảo" -> "Kim cương" trên mọi mặt (game hải tặc dùng Kim cương)
- Bảng thuật ngữ chuan-hoa-dich.py thêm quy tắc; áp cho templates.bin (res/97cec-f0ae6-5f56f,
  byte 10 = 0x76, đã chép assets + docker cp manifest), excel-src (253 ô, 13 workbook biên
  dịch lại, ExcelProbe: lỗi còn lại giống hệt bản trước), ui.bin không có chữ này.
- Web (portal/haitac/market/admin/gm), Go (adapter cửa hàng, admin, gmops, textnorm), tool sinh
  gói/danh mục, PHP cũ, docs: thay theo ba dạng hoa/thường; test Go cập nhật, xanh.
- Seed: game_packages.haitac.sql sinh lại; thêm game_packages.haitac.kim-cuong.sql và
  news.zz-doi-ten-kim-cuong.sql để sửa tên/mô tả gói và tin ĐÃ CÓ trong DB (upsert không đụng
  tên Việt đang lưu).
- templates-bin.py: ghi() bỏ bảng giả _vop cũ trước khi nen() thêm lại.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/excel/release/common.xlsx
+++ b/server/excel/release/common.xlsx
@@ -1063,7 +1063,7 @@
     <t xml:space="preserve">Trợ lực gói quà</t>
   </si>
   <si>
-    <t xml:space="preserve">Trợ lực Bảo bảo Nguyên bảo</t>
+    <t xml:space="preserve">Trợ lực Bảo bảo Kim cương</t>
   </si>
   <si>
     <t xml:space="preserve">Trợ lực tướng Liên sv</t>
@@ -1138,10 +1138,10 @@
     <t xml:space="preserve">Ban đầu ba lô không gian の Đồ cất giữ ba lô</t>
   </si>
   <si>
-    <t xml:space="preserve">Mở rộng tướng ba lô tiêu hao Nguyên bảo cơ sở giá trị</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mở rộng tướng ba lô tiêu hao Nguyên bảo tăng lên giá trị</t>
+    <t xml:space="preserve">Mở rộng tướng ba lô tiêu hao Kim cương cơ sở giá trị</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mở rộng tướng ba lô tiêu hao Kim cương tăng lên giá trị</t>
   </si>
   <si>
     <t xml:space="preserve">Tướng ba lô nhiều nhất khuếch trương cho lượt</t>
@@ -1150,7 +1150,7 @@
     <t xml:space="preserve">Ban đầu ba lô không gian の Thần long</t>
   </si>
   <si>
-    <t xml:space="preserve">Mỗi mua X Lần, tiêu hao Nguyên bảo sẽ tăng lên 1 Lần</t>
+    <t xml:space="preserve">Mỗi mua X Lần, tiêu hao Kim cương sẽ tăng lên 1 Lần</t>
   </si>
   <si>
     <t xml:space="preserve">Một lần mua mở rộng ba lô ngăn chứa số</t>
@@ -1318,13 +1318,13 @@
     <t xml:space="preserve">50#200</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Mệnh cách phó bản 】 Có thù lao mua Nguyên bảo tiêu hao ( Lần lượt tăng lên, cuối cùng ổn định 200)</t>
+    <t xml:space="preserve">【 Mệnh cách phó bản 】 Có thù lao mua Kim cương tiêu hao ( Lần lượt tăng lên, cuối cùng ổn định 200)</t>
   </si>
   <si>
     <t xml:space="preserve">50#200#500</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Mệnh cách tẩy luyện 】 Khóa chặt thuộc tính Nguyên bảo tiêu hao ( Khóa 1 Đầu muốn 50, khóa 2 Đầu muốn 200Cứ thế mà suy ra )</t>
+    <t xml:space="preserve">【 Mệnh cách tẩy luyện 】 Khóa chặt thuộc tính Kim cương tiêu hao ( Khóa 1 Đầu muốn 50, khóa 2 Đầu muốn 200Cứ thế mà suy ra )</t>
   </si>
   <si>
     <t xml:space="preserve">12</t>
@@ -1345,7 +1345,7 @@
     <t xml:space="preserve">36 trọng thiên tướng đóng giữ gia tốc miễn phí lượt</t>
   </si>
   <si>
-    <t xml:space="preserve">36 trọng thiên tướng đóng giữ gia tốc Nguyên bảo mua lượt</t>
+    <t xml:space="preserve">36 trọng thiên tướng đóng giữ gia tốc Kim cương mua lượt</t>
   </si>
   <si>
     <t xml:space="preserve">2</t>
@@ -1357,7 +1357,7 @@
     <t xml:space="preserve">50#100#200</t>
   </si>
   <si>
-    <t xml:space="preserve">36 trọng thiên đóng giữ gia tốc có thù lao mua Nguyên bảo tiêu hao ( Lượt cùng phí tổn )</t>
+    <t xml:space="preserve">36 trọng thiên đóng giữ gia tốc có thù lao mua Kim cương tiêu hao ( Lượt cùng phí tổn )</t>
   </si>
   <si>
     <t xml:space="preserve">1000000</t>
@@ -1480,7 +1480,7 @@
     <t xml:space="preserve">【 Tỉ ấn 】 Vượt phục tỉ ấn hoạt động tiêu hao tỉ lệ</t>
   </si>
   <si>
-    <t xml:space="preserve">Wechat chia sẻ thủ xông trả về Nguyên bảo hệ số</t>
+    <t xml:space="preserve">Wechat chia sẻ thủ xông trả về Kim cương hệ số</t>
   </si>
   <si>
     <t xml:space="preserve">Wechat chia sẻ thủ xông trả về hữu nghị điểm hệ số</t>
@@ -1618,7 +1618,7 @@
     <t xml:space="preserve">【 Nhanh chóng tác chiến 】 Nhanh chóng tác chiến có thể nhận được treo máy thời gian ( Phút )</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Nhanh chóng tác chiến 】 Có thù lao mua Nguyên bảo tiêu hao ( Lần lượt tăng lên, cuối cùng ổn định 200)</t>
+    <t xml:space="preserve">【 Nhanh chóng tác chiến 】 Có thù lao mua Kim cương tiêu hao ( Lần lượt tăng lên, cuối cùng ổn định 200)</t>
   </si>
   <si>
     <t xml:space="preserve">0.5</t>
@@ -1933,7 +1933,7 @@
     <t xml:space="preserve">【 Treo thưởng nhiệm vụ 】 Sử dụng đạo cụ đổi mới tiêu hao</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Treo thưởng nhiệm vụ 】 Sử dụng Nguyên bảo đổi mới giá cả m1</t>
+    <t xml:space="preserve">【 Treo thưởng nhiệm vụ 】 Sử dụng Kim cương đổi mới giá cả m1</t>
   </si>
   <si>
     <t xml:space="preserve">【 Treo thưởng nhiệm vụ 】 Mỗi lần đổi mới ra nhiệm vụ số lượng</t>
@@ -2077,7 +2077,7 @@
     <t xml:space="preserve">【 Cá nhân không gian 】 Sửa chữa danh tự miễn phí lượt</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Cá nhân không gian 】 Sửa chữa danh tự Nguyên bảo tiêu hao</t>
+    <t xml:space="preserve">【 Cá nhân không gian 】 Sửa chữa danh tự Kim cương tiêu hao</t>
   </si>
   <si>
     <t xml:space="preserve">【 Cá nhân không gian 】 Nhân vật chính danh tự ít nhất số lượng từ</t>
@@ -2116,7 +2116,7 @@
     <t xml:space="preserve">【 Nạp tiền phúc lợi 】 Nhanh chóng tác chiến quỹ ngân sách giá ưu đãi cách (RMB)( Kích hoạt nhanh chóng tác chiến đặc quyền về sau mua giá cả )</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Nạp tiền phúc lợi 】 Thủ mạo xưng gấp đôi Nguyên bảo đổi mới phiên bản hào ( Việt Nam bản công năngThay đổi sau đổi mới người chơi trên thân trạng thái )</t>
+    <t xml:space="preserve">【 Nạp tiền phúc lợi 】 Thủ mạo xưng gấp đôi Kim cương đổi mới phiên bản hào ( Việt Nam bản công năngThay đổi sau đổi mới người chơi trên thân trạng thái )</t>
   </si>
   <si>
     <t xml:space="preserve">【 Nạp tiền phúc lợi 】 Tuần hạn mua thiết lập lại phiên bản hào ( Hàn Quốc công năngThay đổi sau thiết lập lại tuần hạn mua mua lượt )</t>
@@ -2161,13 +2161,13 @@
     <t xml:space="preserve">Mạo hiểm treo máy địa đồ</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Chiến lệnh 】 Dư thừa chiến lệnh điểm tích lũy chuyển đổi Nguyên bảo tỉ lệ (1 Điểm tích lũy = 0.1 Nguyên bảo )</t>
+    <t xml:space="preserve">【 Chiến lệnh 】 Dư thừa chiến lệnh điểm tích lũy chuyển đổi Kim cương tỉ lệ (1 Điểm tích lũy = 0.1 Kim cương )</t>
   </si>
   <si>
     <t xml:space="preserve">【 Chiến lệnh 】 Mỗi tuần nhiệm vụ tiếp tục số trời</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Chiến lệnh 】 Đơn lần mua điểm tích lũy Nguyên bảo tiêu hao</t>
+    <t xml:space="preserve">【 Chiến lệnh 】 Đơn lần mua điểm tích lũy Kim cương tiêu hao</t>
   </si>
   <si>
     <t xml:space="preserve">【 Chiến lệnh 】 Đơn lần mua điểm tích lũy tăng lên</t>
@@ -2182,7 +2182,7 @@
     <t xml:space="preserve">【 Cây bồ đề 】 Mỗi ngày có thể mua mua tưới nước lượt</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Cây bồ đề 】 Mua tưới nước lượt Nguyên bảo tiêu hao</t>
+    <t xml:space="preserve">【 Cây bồ đề 】 Mua tưới nước lượt Kim cương tiêu hao</t>
   </si>
   <si>
     <t xml:space="preserve">【 Cây bồ đề 】 Tưới nước hậu quả thực gia tốc giờ số</t>
@@ -2194,7 +2194,7 @@
     <t xml:space="preserve">【 Cây bồ đề 】 Mỗi ngày có thể mua mua bón phân lượt</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Cây bồ đề 】 Bón phân Nguyên bảo tiêu hao</t>
+    <t xml:space="preserve">【 Cây bồ đề 】 Bón phân Kim cương tiêu hao</t>
   </si>
   <si>
     <t xml:space="preserve">【 Cây bồ đề 】 Bón phân gia tăng kinh nghiệm</t>
@@ -2281,7 +2281,7 @@
     <t xml:space="preserve">【 Thiên giới mê cung 】 Kéo lấy chân nhân chiến lực ba động tỉ lệ</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Thiên giới mê cung chiến lệnh 】 Mua chiến lệnh Nguyên bảo tiêu hao</t>
+    <t xml:space="preserve">【 Thiên giới mê cung chiến lệnh 】 Mua chiến lệnh Kim cương tiêu hao</t>
   </si>
   <si>
     <t xml:space="preserve">【 Thiên giới mê cung chiến lệnh 】 Đơn lần mua điểm tích lũy gia tăng</t>
@@ -2293,7 +2293,7 @@
     <t xml:space="preserve">100#200#300#400#500</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Tướng trùng sinh 】 Một lần trùng sinh Nguyên bảo tiêu hao</t>
+    <t xml:space="preserve">【 Tướng trùng sinh 】 Một lần trùng sinh Kim cương tiêu hao</t>
   </si>
   <si>
     <t xml:space="preserve">【 Tướng trùng sinh 】 Trùng sinh miễn phí số trời ( Khai phục trước 7 Trời )</t>
@@ -2332,7 +2332,7 @@
     <t xml:space="preserve">【 Thế giới BOSS】 Mỗi ngày có thể mua mua khiêu chiến lượt</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Thế giới BOSS】 Mua lượt Nguyên bảo tiêu hao</t>
+    <t xml:space="preserve">【 Thế giới BOSS】 Mua lượt Kim cương tiêu hao</t>
   </si>
   <si>
     <t xml:space="preserve">【 Hoan độ Trung thu 】 Mỗi ngày miễn phí khiêu chiến lượt</t>
@@ -2341,7 +2341,7 @@
     <t xml:space="preserve">【 Hoan độ Trung thu 】 Mỗi ngày có thể mua mua khiêu chiến lượt</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Hoan độ Trung thu 】 Mua lượt Nguyên bảo tiêu hao</t>
+    <t xml:space="preserve">【 Hoan độ Trung thu 】 Mua lượt Kim cương tiêu hao</t>
   </si>
   <si>
     <t xml:space="preserve">3:1000016:1#3:1000011:1#3:100001:1</t>
@@ -2383,13 +2383,13 @@
     <t xml:space="preserve">Tiên Khí đạt tới XX Tinh phân giải có nhắc nhở</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Kỳ nghỉ hè đại tác chiến 】 Dư thừa điểm tích lũy chuyển đổi Nguyên bảo tỉ lệ (1 Điểm tích lũy = 0.1 Nguyên bảo )</t>
+    <t xml:space="preserve">【 Kỳ nghỉ hè đại tác chiến 】 Dư thừa điểm tích lũy chuyển đổi Kim cương tỉ lệ (1 Điểm tích lũy = 0.1 Kim cương )</t>
   </si>
   <si>
     <t xml:space="preserve">【 Kỳ nghỉ hè đại tác chiến 】 Mỗi tuần nhiệm vụ tiếp tục số trời</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Kỳ nghỉ hè đại tác chiến 】 Đơn lần mua điểm tích lũy Nguyên bảo tiêu hao</t>
+    <t xml:space="preserve">【 Kỳ nghỉ hè đại tác chiến 】 Đơn lần mua điểm tích lũy Kim cương tiêu hao</t>
   </si>
   <si>
     <t xml:space="preserve">【 Kỳ nghỉ hè đại tác chiến 】 Đơn lần mua điểm tích lũy tăng lên</t>
@@ -2605,7 +2605,7 @@
     <t xml:space="preserve">0.08</t>
   </si>
   <si>
-    <t xml:space="preserve">【 Đỉnh phong biết võ 】 Cạnh đoán hối đoái tỉ lệ 1 Nguyên bảo đổi N Võ Thần điểm tích lũy</t>
+    <t xml:space="preserve">【 Đỉnh phong biết võ 】 Cạnh đoán hối đoái tỉ lệ 1 Kim cương đổi N Võ Thần điểm tích lũy</t>
   </si>
   <si>
     <t xml:space="preserve">【 Đỉnh phong biết võ 】 Một cái quán quân bị kính ngưỡng đầu số hạn mức cao nhất</t>

</xml_diff>